<commit_message>
feat: UX and Dashboard metrics, Premium Landing Page, Schedules, and Auth Persistence
</commit_message>
<xml_diff>
--- a/carteira A.xlsx
+++ b/carteira A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasdematos/Desktop/ARVO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD588E3-4EAF-3A4D-8A49-7F060507BEAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3741FC0E-ED68-974E-A4A6-0988379E98CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40" yWindow="680" windowWidth="26500" windowHeight="18040" firstSheet="3" activeTab="9" xr2:uid="{F4717258-1541-41AD-9103-EA3611101638}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5560" uniqueCount="2202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5560" uniqueCount="2203">
   <si>
     <t>Carteira A</t>
   </si>
@@ -8052,6 +8052,9 @@
   </si>
   <si>
     <t>% SobreIPCA</t>
+  </si>
+  <si>
+    <t>Kinea Debêntures Incentivadas FIRF/Itaú Debêntures Incentivadas CDI/ARX Hedge Master FI Infra Renda Fixa/ARX Hedge FIC Incentivado Financeiro em Infra RF RL</t>
   </si>
 </sst>
 </file>
@@ -12378,7 +12381,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="72" t="s">
-        <v>1466</v>
+        <v>2202</v>
       </c>
       <c r="B6" s="74">
         <v>7.4999999999999997E-2</v>
@@ -14075,7 +14078,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE7B6B8-3383-0848-B7C0-5CA005D84B68}">
-  <dimension ref="A1:P77"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
@@ -16066,6 +16069,30 @@
       <c r="D77" s="102">
         <v>111.43</v>
       </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="72"/>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" s="72"/>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="75"/>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="72"/>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="72"/>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="72"/>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" s="72"/>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -47109,7 +47136,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="72" t="s">
-        <v>1447</v>
+        <v>2198</v>
       </c>
       <c r="B4" s="74">
         <v>0.04</v>
@@ -47217,7 +47244,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="72" t="s">
-        <v>2097</v>
+        <v>1979</v>
       </c>
       <c r="B10" s="74">
         <v>0.04</v>

</xml_diff>